<commit_message>
feat: correções nos campos do handlebars
</commit_message>
<xml_diff>
--- a/public/files/planilha.xlsx
+++ b/public/files/planilha.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="41">
   <si>
     <t>Mestrados</t>
   </si>
@@ -62,25 +62,25 @@
     <t>Observações</t>
   </si>
   <si>
-    <t>Jon</t>
-  </si>
-  <si>
-    <t>jon@email.com</t>
+    <t>Candidato teste</t>
+  </si>
+  <si>
+    <t>francisco.junior@icomp.ufam.edu.br</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Mestrado</t>
   </si>
   <si>
+    <t>teste teste</t>
+  </si>
+  <si>
     <t>Doutorados</t>
-  </si>
-  <si>
-    <t>Jane</t>
-  </si>
-  <si>
-    <t>jane@email.com</t>
-  </si>
-  <si>
-    <t>Doutorado</t>
   </si>
   <si>
     <t>Nota Final</t>
@@ -536,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="40" customWidth="1"/>
@@ -609,20 +609,35 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="C3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3" t="b">
+        <v>0</v>
+      </c>
       <c r="G3" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -682,17 +697,6 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:N1"/>
@@ -705,7 +709,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -740,7 +744,7 @@
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -754,14 +758,6 @@
       </c>
       <c r="C5" s="2" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="3">
-        <f>=Candidato!B:B</f>
       </c>
     </row>
   </sheetData>
@@ -776,7 +772,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="40" customWidth="1"/>
@@ -819,7 +815,7 @@
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -841,14 +837,6 @@
       </c>
       <c r="E5" s="2" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="3">
-        <f>=SUM(B6:D6)</f>
       </c>
     </row>
   </sheetData>
@@ -863,7 +851,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -911,7 +899,7 @@
     <row r="3" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>31</v>
@@ -948,7 +936,7 @@
     </row>
     <row r="5" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B5"/>
       <c r="C5"/>
@@ -985,7 +973,7 @@
     <row r="7" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>31</v>
@@ -1007,18 +995,6 @@
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I8" s="3">
-        <f>=IF(SUM(B8:E8)&gt;30,30,SUM(B8:E8)) + IF(SUM(F8:H8)&gt;70,70,SUM(F8:H8)</f>
-      </c>
-      <c r="J8" s="3" t="str">
-        <f>=5+((5*I8)/100)</f>
-        <v>5</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1042,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1096,7 +1072,7 @@
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -1118,25 +1094,6 @@
       </c>
       <c r="E5" s="2" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="3">
-        <f>=Provas!C:C</f>
-      </c>
-      <c r="C6" s="3">
-        <f>=Propostas!E:E</f>
-      </c>
-      <c r="D6" s="3" t="str">
-        <f>=Titulos!I:I</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="str">
-        <f>AVERAGE(B2:D2)</f>
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: alterações de rotas em recomendação de candidato
</commit_message>
<xml_diff>
--- a/public/files/planilha.xlsx
+++ b/public/files/planilha.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="42">
   <si>
     <t>Mestrados</t>
   </si>
@@ -62,7 +62,10 @@
     <t>Observações</t>
   </si>
   <si>
-    <t>Candidato teste</t>
+    <t>Doutorados</t>
+  </si>
+  <si>
+    <t>Francisco</t>
   </si>
   <si>
     <t>francisco.junior@icomp.ufam.edu.br</t>
@@ -74,40 +77,40 @@
     <t/>
   </si>
   <si>
+    <t>Doutorado</t>
+  </si>
+  <si>
+    <t>teste teste</t>
+  </si>
+  <si>
+    <t>Nota Final</t>
+  </si>
+  <si>
+    <t>Avaliador 1</t>
+  </si>
+  <si>
+    <t>Avaliador 2</t>
+  </si>
+  <si>
+    <t>Avaliador 3</t>
+  </si>
+  <si>
+    <t>Media Final</t>
+  </si>
+  <si>
+    <t>Atividades Curriculares e Extracurriculares (30 pontos)</t>
+  </si>
+  <si>
+    <t>Publicações (70 pontos)</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>NAC</t>
+  </si>
+  <si>
     <t>Mestrado</t>
-  </si>
-  <si>
-    <t>teste teste</t>
-  </si>
-  <si>
-    <t>Doutorados</t>
-  </si>
-  <si>
-    <t>Nota Final</t>
-  </si>
-  <si>
-    <t>Avaliador 1</t>
-  </si>
-  <si>
-    <t>Avaliador 2</t>
-  </si>
-  <si>
-    <t>Avaliador 3</t>
-  </si>
-  <si>
-    <t>Media Final</t>
-  </si>
-  <si>
-    <t>Atividades Curriculares e Extracurriculares (30 pontos)</t>
-  </si>
-  <si>
-    <t>Publicações (70 pontos)</t>
-  </si>
-  <si>
-    <t>Nota</t>
-  </si>
-  <si>
-    <t>NAC</t>
   </si>
   <si>
     <t>Estágio, Extensão e monitoria</t>
@@ -609,98 +612,98 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" ht="35" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3"/>
+      <c r="K3"/>
+      <c r="L3"/>
+      <c r="M3"/>
+      <c r="N3"/>
+    </row>
+    <row r="4" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="3">
+      <c r="C5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="3">
         <v>1</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="3" t="b">
+      <c r="E5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" ht="35" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="K5" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-      <c r="J4"/>
-      <c r="K4"/>
-      <c r="L4"/>
-      <c r="M4"/>
-      <c r="N4"/>
-    </row>
-    <row r="5" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A3:N3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -709,7 +712,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -734,17 +737,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="3">
-        <f>=Candidato!B:B</f>
-      </c>
-    </row>
     <row r="4" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -758,6 +753,14 @@
       </c>
       <c r="C5" s="2" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3">
+        <f>=Candidato!B:B</f>
       </c>
     </row>
   </sheetData>
@@ -772,7 +775,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="40" customWidth="1"/>
@@ -805,17 +808,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="3">
-        <f>=SUM(B3:D3)</f>
-      </c>
-    </row>
     <row r="4" ht="35" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -837,6 +832,14 @@
       </c>
       <c r="E5" s="2" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="3">
+        <f>=SUM(B6:D6)</f>
       </c>
     </row>
   </sheetData>
@@ -851,7 +854,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -899,44 +902,32 @@
     <row r="3" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="4" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="3">
-        <f>=IF(SUM(B4:E4)&gt;30,30,SUM(B4:E4)) + IF(SUM(F4:H4)&gt;70,70,SUM(F4:H4)</f>
-      </c>
-      <c r="J4" s="3" t="str">
-        <f>=5+((5*I4)/100)</f>
-        <v>5</v>
-      </c>
-    </row>
     <row r="5" ht="35" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B5"/>
       <c r="C5"/>
@@ -973,28 +964,40 @@
     <row r="7" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="3">
+        <f>=IF(SUM(B8:E8)&gt;30,30,SUM(B8:E8)) + IF(SUM(F8:H8)&gt;70,70,SUM(F8:H8)</f>
+      </c>
+      <c r="J8" s="3" t="str">
+        <f>=5+((5*I8)/100)</f>
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1018,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1039,40 +1042,21 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="3">
-        <f>=Provas!C:C</f>
-      </c>
-      <c r="C3" s="3">
-        <f>=Propostas!E:E</f>
-      </c>
-      <c r="D3" s="3" t="str">
-        <f>=Titulos!I:I</f>
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="str">
-        <f>AVERAGE(B2:D2)</f>
-        <v>0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -1084,16 +1068,35 @@
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3">
+        <f>=Provas!C:C</f>
+      </c>
+      <c r="C6" s="3">
+        <f>=Propostas!E:E</f>
+      </c>
+      <c r="D6" s="3" t="str">
+        <f>=Titulos!I:I</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="str">
+        <f>AVERAGE(B2:D2)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>